<commit_message>
feat(members): import VPDive groups and price active members
- Added the optional « Organisation » column to `members.Parse` as `Member.Organisation`, sealed in the new `members.organisation` column (migration `0014_member_organisation.sql`).
- Renamed the `seasons` cell reader to `list`, shared by « Année(s) » and « Organisation », and introduced `Store.openInto` for optional sealed columns.
- Exposed the groups as `organisation` in the `find_member` candidates and the `<demande>` requester, through `candidateOf`.
- Added the « Membres actifs » plans and guest products to the resolver procedure of the fiche `tarification`, with three new anomalies.
</commit_message>
<xml_diff>
--- a/testdata/fixtures/members_duplicate_email.xlsx
+++ b/testdata/fixtures/members_duplicate_email.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t xml:space="preserve">Liste des membres Club de plongée d'exemple</t>
   </si>
@@ -71,6 +71,9 @@
   </si>
   <si>
     <t xml:space="preserve">Année(s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organisation</t>
   </si>
   <si>
     <t xml:space="preserve">Mme</t>
@@ -218,55 +221,58 @@
       <c r="W4" t="s">
         <v>20</v>
       </c>
+      <c r="X4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="M5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="U5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="V5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W5">
         <v>2026</v>
@@ -277,49 +283,49 @@
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>37</v>
+      </c>
+      <c r="I6" t="s">
+        <v>25</v>
+      </c>
+      <c r="J6" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" t="s">
+        <v>27</v>
+      </c>
+      <c r="L6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N6" t="s">
+        <v>30</v>
+      </c>
+      <c r="P6" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>32</v>
+      </c>
+      <c r="R6" t="s">
+        <v>33</v>
+      </c>
+      <c r="S6" t="s">
+        <v>34</v>
+      </c>
+      <c r="U6" t="s">
+        <v>31</v>
+      </c>
+      <c r="V6" t="s">
         <v>35</v>
-      </c>
-      <c r="G6" t="s">
-        <v>36</v>
-      </c>
-      <c r="I6" t="s">
-        <v>24</v>
-      </c>
-      <c r="J6" t="s">
-        <v>37</v>
-      </c>
-      <c r="K6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L6" t="s">
-        <v>27</v>
-      </c>
-      <c r="M6" t="s">
-        <v>28</v>
-      </c>
-      <c r="N6" t="s">
-        <v>29</v>
-      </c>
-      <c r="P6" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>31</v>
-      </c>
-      <c r="R6" t="s">
-        <v>32</v>
-      </c>
-      <c r="S6" t="s">
-        <v>33</v>
-      </c>
-      <c r="U6" t="s">
-        <v>30</v>
-      </c>
-      <c r="V6" t="s">
-        <v>34</v>
       </c>
       <c r="W6">
         <v>2026</v>
@@ -330,49 +336,49 @@
         <v>3</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="M7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="U7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="V7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W7">
         <v>2026</v>

</xml_diff>